<commit_message>
Align level tables with marine proposal columns (type, term_localName, label, external url, parent unit name)
</commit_message>
<xml_diff>
--- a/terrestrial/Towards_SDS/Level1_SDS-aligned.xlsx
+++ b/terrestrial/Towards_SDS/Level1_SDS-aligned.xlsx
@@ -91,8 +91,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -470,209 +473,290 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13.86" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="13.86" customWidth="1" min="2" max="2"/>
     <col width="19.86" customWidth="1" min="3" max="3"/>
     <col width="18.57" customWidth="1" min="5" max="5"/>
     <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="18.57" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
           <t>Id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Local_name</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Full_name</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>term_localName/
+controlled_value_string</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>label</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>external url</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>parent unit name</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>Change according to page 9</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>Exchange notes</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>Definition</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="n">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>concept</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="C2" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="D2" s="5" t="inlineStr">
         <is>
           <t>Europe</t>
         </is>
       </c>
-      <c r="D2" s="4" t="n"/>
-      <c r="E2" s="4" t="n"/>
-      <c r="F2" s="4" t="n"/>
+      <c r="E2" s="5" t="n"/>
+      <c r="F2" s="5" t="n"/>
+      <c r="G2" s="5" t="n"/>
+      <c r="H2" s="5" t="n"/>
+      <c r="I2" s="5" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="n">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>concept</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>Africa</t>
         </is>
       </c>
-      <c r="D3" s="4" t="n"/>
-      <c r="E3" s="4" t="n"/>
-      <c r="F3" s="4" t="n"/>
+      <c r="E3" s="5" t="n"/>
+      <c r="F3" s="5" t="n"/>
+      <c r="G3" s="5" t="n"/>
+      <c r="H3" s="5" t="n"/>
+      <c r="I3" s="5" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="n">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>concept</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>Asia-Temperate</t>
         </is>
       </c>
-      <c r="D4" s="4" t="n"/>
-      <c r="E4" s="4" t="n"/>
-      <c r="F4" s="4" t="n"/>
+      <c r="E4" s="5" t="n"/>
+      <c r="F4" s="5" t="n"/>
+      <c r="G4" s="5" t="n"/>
+      <c r="H4" s="5" t="n"/>
+      <c r="I4" s="5" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="n">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>concept</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>Asia-Tropical</t>
         </is>
       </c>
-      <c r="D5" s="4" t="n"/>
-      <c r="E5" s="4" t="n"/>
-      <c r="F5" s="4" t="n"/>
+      <c r="E5" s="5" t="n"/>
+      <c r="F5" s="5" t="n"/>
+      <c r="G5" s="5" t="n"/>
+      <c r="H5" s="5" t="n"/>
+      <c r="I5" s="5" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="n">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>concept</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>Australasia</t>
         </is>
       </c>
-      <c r="D6" s="4" t="n"/>
-      <c r="E6" s="4" t="n"/>
-      <c r="F6" s="4" t="n"/>
+      <c r="E6" s="5" t="n"/>
+      <c r="F6" s="5" t="n"/>
+      <c r="G6" s="5" t="n"/>
+      <c r="H6" s="5" t="n"/>
+      <c r="I6" s="5" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="n">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>concept</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>Pacific</t>
         </is>
       </c>
-      <c r="D7" s="4" t="n"/>
-      <c r="E7" s="4" t="n"/>
-      <c r="F7" s="4" t="n"/>
+      <c r="E7" s="5" t="n"/>
+      <c r="F7" s="5" t="n"/>
+      <c r="G7" s="5" t="n"/>
+      <c r="H7" s="5" t="n"/>
+      <c r="I7" s="5" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="n">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>concept</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>Northern America</t>
         </is>
       </c>
-      <c r="D8" s="4" t="n"/>
-      <c r="E8" s="4" t="n"/>
-      <c r="F8" s="4" t="n"/>
+      <c r="E8" s="5" t="n"/>
+      <c r="F8" s="5" t="n"/>
+      <c r="G8" s="5" t="n"/>
+      <c r="H8" s="5" t="n"/>
+      <c r="I8" s="5" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="n">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>concept</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>Southern America</t>
         </is>
       </c>
-      <c r="D9" s="4" t="n"/>
-      <c r="E9" s="4" t="n"/>
-      <c r="F9" s="4" t="n"/>
+      <c r="E9" s="5" t="n"/>
+      <c r="F9" s="5" t="n"/>
+      <c r="G9" s="5" t="n"/>
+      <c r="H9" s="5" t="n"/>
+      <c r="I9" s="5" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="n">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>concept</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>Antarctic</t>
         </is>
       </c>
-      <c r="D10" s="4" t="n"/>
-      <c r="E10" s="4" t="n"/>
-      <c r="F10" s="4" t="n"/>
+      <c r="E10" s="5" t="n"/>
+      <c r="F10" s="5" t="n"/>
+      <c r="G10" s="5" t="n"/>
+      <c r="H10" s="5" t="n"/>
+      <c r="I10" s="5" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Populate Definition column for all units; fix CZE/SK ISO code swap
</commit_message>
<xml_diff>
--- a/terrestrial/Towards_SDS/Level1_SDS-aligned.xlsx
+++ b/terrestrial/Towards_SDS/Level1_SDS-aligned.xlsx
@@ -556,7 +556,11 @@
       <c r="F2" s="5" t="n"/>
       <c r="G2" s="5" t="n"/>
       <c r="H2" s="5" t="n"/>
-      <c r="I2" s="5" t="n"/>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>The territory comprising 10, 11, 12, 13, and 14.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -581,7 +585,11 @@
       <c r="F3" s="5" t="n"/>
       <c r="G3" s="5" t="n"/>
       <c r="H3" s="5" t="n"/>
-      <c r="I3" s="5" t="n"/>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>The territory comprising 20, 21, 22, 23, 24, 25, 26, 27, 28, and 29.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -606,7 +614,11 @@
       <c r="F4" s="5" t="n"/>
       <c r="G4" s="5" t="n"/>
       <c r="H4" s="5" t="n"/>
-      <c r="I4" s="5" t="n"/>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>The territory comprising 30, 31, 32, 33, 34, 35, 36, 37, and 38.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -631,7 +643,11 @@
       <c r="F5" s="5" t="n"/>
       <c r="G5" s="5" t="n"/>
       <c r="H5" s="5" t="n"/>
-      <c r="I5" s="5" t="n"/>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>The territory comprising 40, 41, 42, and 43.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -656,7 +672,11 @@
       <c r="F6" s="5" t="n"/>
       <c r="G6" s="5" t="n"/>
       <c r="H6" s="5" t="n"/>
-      <c r="I6" s="5" t="n"/>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>The territory comprising 50 and 51.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -681,7 +701,11 @@
       <c r="F7" s="5" t="n"/>
       <c r="G7" s="5" t="n"/>
       <c r="H7" s="5" t="n"/>
-      <c r="I7" s="5" t="n"/>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>The territory comprising 60, 61, 62, and 63.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -706,7 +730,11 @@
       <c r="F8" s="5" t="n"/>
       <c r="G8" s="5" t="n"/>
       <c r="H8" s="5" t="n"/>
-      <c r="I8" s="5" t="n"/>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>The territory comprising 70, 71, 72, 73, 74, 75, 76, 77, 78, and 79.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -731,7 +759,11 @@
       <c r="F9" s="5" t="n"/>
       <c r="G9" s="5" t="n"/>
       <c r="H9" s="5" t="n"/>
-      <c r="I9" s="5" t="n"/>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>The territory comprising 80, 81, 82, 83, 84, and 85.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -756,7 +788,11 @@
       <c r="F10" s="5" t="n"/>
       <c r="G10" s="5" t="n"/>
       <c r="H10" s="5" t="n"/>
-      <c r="I10" s="5" t="n"/>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>The territory comprising 90 and 91.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>